<commit_message>
9th june - 7 PM
working code
</commit_message>
<xml_diff>
--- a/Ref docs/Configuration/Dropdown/NEw configs.xlsx
+++ b/Ref docs/Configuration/Dropdown/NEw configs.xlsx
@@ -8,20 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rockwellautomation-my.sharepoint.com/personal/anjana_sharma_rockwellautomation_com/Documents/Anjana Sharma - All Important Documents/1. My work/RA Work/AM-APP/Ref docs/Configuration/Dropdown/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{B726ADD6-1307-4B66-BB01-1592C31C5EDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D7D8D49-AA02-48EA-8FC6-D746BA1D578E}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{B726ADD6-1307-4B66-BB01-1592C31C5EDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{304E69F7-46B2-465E-815B-6381F02B2D12}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Configurations" sheetId="1" r:id="rId1"/>
-    <sheet name="Available Link Targets" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
   <si>
     <t>Configuration Type</t>
   </si>
@@ -38,73 +37,16 @@
     <t>Linked To (Labels)</t>
   </si>
   <si>
-    <t>blue</t>
-  </si>
-  <si>
-    <t>request_processing_status_field</t>
-  </si>
-  <si>
-    <t>Processing Status dropdown</t>
-  </si>
-  <si>
-    <t>green</t>
-  </si>
-  <si>
-    <t>request_overall_status_field</t>
-  </si>
-  <si>
-    <t>Overall Status dropdown</t>
-  </si>
-  <si>
-    <t>ra_process_account_anchor_field</t>
-  </si>
-  <si>
-    <t>Account Anchor allocation</t>
-  </si>
-  <si>
-    <t>Link Target ID</t>
-  </si>
-  <si>
-    <t>Label</t>
-  </si>
-  <si>
-    <t>Module</t>
-  </si>
-  <si>
-    <t>Request Management</t>
-  </si>
-  <si>
-    <t>RA Process</t>
-  </si>
-  <si>
-    <t>resource_skill_field</t>
-  </si>
-  <si>
-    <t>Resource Skill dropdown</t>
-  </si>
-  <si>
-    <t>Resource Details</t>
-  </si>
-  <si>
-    <t>resource_designation_field</t>
-  </si>
-  <si>
-    <t>Resource Designation dropdown</t>
-  </si>
-  <si>
-    <t>request_type_field</t>
-  </si>
-  <si>
-    <t>Request Type dropdown</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test value 1 </t>
-  </si>
-  <si>
-    <t>Test value 2</t>
+    <t>PCTeam</t>
+  </si>
+  <si>
+    <t>Rajashekhar</t>
+  </si>
+  <si>
+    <t>Glasteena</t>
+  </si>
+  <si>
+    <t>Manjunath</t>
   </si>
 </sst>
 </file>
@@ -481,7 +423,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="30.83203125" customWidth="1"/>
@@ -509,124 +451,32 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E1 C2" numberStoredAsText="1"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="2" width="40.83203125" customWidth="1"/>
-    <col min="3" max="3" width="25.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:C7" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:E1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>